<commit_message>
update profiles and main func
</commit_message>
<xml_diff>
--- a/feeder 5/RepDays.xlsx
+++ b/feeder 5/RepDays.xlsx
@@ -442,42 +442,42 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>81</v>
+        <v>122</v>
       </c>
       <c r="B2" t="n">
-        <v>0.06346325334823852</v>
+        <v>0.173115900563808</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>91</v>
+        <v>126</v>
       </c>
       <c r="B3" t="n">
-        <v>0.1280422590634022</v>
+        <v>0.2663411593687789</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>122</v>
+        <v>243</v>
       </c>
       <c r="B4" t="n">
-        <v>0.3396295291049402</v>
+        <v>0.07214007476005649</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>133</v>
+        <v>279</v>
       </c>
       <c r="B5" t="n">
-        <v>0.1232736320715953</v>
+        <v>0.2965235005405597</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>175</v>
+        <v>308</v>
       </c>
       <c r="B6" t="n">
-        <v>0.3455913264118234</v>
+        <v>0.1918793647667969</v>
       </c>
     </row>
   </sheetData>

</xml_diff>